<commit_message>
Actualización a V6.0: Optimizaciones de scraping extremo, nueva documentación y limpieza de archivos
</commit_message>
<xml_diff>
--- a/PLANTILLA CON INFORME.xlsx
+++ b/PLANTILLA CON INFORME.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\DESCARGAS\PROYECTOS\PROYECTO PREGUNTAS GOOGLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19946233-0805-4926-902B-7321D81FBE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481FF363-95F8-4CB3-8EC7-EF13300FA1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7108" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7048" uniqueCount="396">
   <si>
     <t>Analisis de keyword: Internet claro</t>
   </si>
@@ -1172,15 +1172,9 @@
     <t>Propuestas de artículos + títulos SEO</t>
   </si>
   <si>
-    <t>Enfoque:</t>
-  </si>
-  <si>
     <t>Usuarios buscando cuál plan contratar, precios actuales y beneficios frente a otros operadores.</t>
   </si>
   <si>
-    <t>Títulos:</t>
-  </si>
-  <si>
     <t>Internet Claro: precios y planes para hogar en 2026</t>
   </si>
   <si>
@@ -1196,9 +1190,6 @@
     <t>Internet Claro hogar: comparación de planes y cobertura</t>
   </si>
   <si>
-    <t>Ideas de subtítulos:</t>
-  </si>
-  <si>
     <t>Qué incluye cada plan</t>
   </si>
   <si>
@@ -1209,182 +1200,6 @@
   </si>
   <si>
     <t>Cómo elegir el mejor plan según tu uso</t>
-  </si>
-  <si>
-    <t>2. Artículo sobre fallas y soluciones</t>
-  </si>
-  <si>
-    <t>Alta intención de búsqueda por problemas técnicos y soporte.</t>
-  </si>
-  <si>
-    <t>Internet Claro con fallas: causas y soluciones rápidas</t>
-  </si>
-  <si>
-    <t>¿Por qué está fallando el Internet Claro hoy?</t>
-  </si>
-  <si>
-    <t>Cómo solucionar problemas frecuentes de Internet Claro</t>
-  </si>
-  <si>
-    <t>Internet Claro lento: qué hacer y cómo reportarlo</t>
-  </si>
-  <si>
-    <t>Fallas de Internet Claro: señales de daño y posibles soluciones</t>
-  </si>
-  <si>
-    <t>Reinicio correcto del módem</t>
-  </si>
-  <si>
-    <t>Cómo saber si hay caída nacional</t>
-  </si>
-  <si>
-    <t>Cuándo llamar a soporte</t>
-  </si>
-  <si>
-    <t>Problemas comunes en fibra óptica</t>
-  </si>
-  <si>
-    <t>3. Comparativo con otros operadores</t>
-  </si>
-  <si>
-    <t>Contenido evergreen con fuerte potencial SEO.</t>
-  </si>
-  <si>
-    <t>Internet Claro vs Movistar: diferencias y precios</t>
-  </si>
-  <si>
-    <t>¿Internet Claro o Tigo? Comparativa completa</t>
-  </si>
-  <si>
-    <t>Qué operador tiene mejor internet en Colombia en 2026</t>
-  </si>
-  <si>
-    <t>Internet Claro frente a ETB: velocidad, estabilidad y cobertura</t>
-  </si>
-  <si>
-    <t>Claro internet hogar: ventajas y desventajas frente a la competencia</t>
-  </si>
-  <si>
-    <t>Velocidad promedio</t>
-  </si>
-  <si>
-    <t>Estabilidad de conexión</t>
-  </si>
-  <si>
-    <t>Cobertura en ciudades</t>
-  </si>
-  <si>
-    <t>Atención al cliente</t>
-  </si>
-  <si>
-    <t>Precio por megas</t>
-  </si>
-  <si>
-    <t>4. Artículo sobre canales de atención y soporte</t>
-  </si>
-  <si>
-    <t>Basado en búsquedas relacionadas de “canales”.</t>
-  </si>
-  <si>
-    <t>Canales de atención de Internet Claro: cómo contactar soporte</t>
-  </si>
-  <si>
-    <t>Internet Claro: líneas, WhatsApp y canales de ayuda</t>
-  </si>
-  <si>
-    <t>Cómo comunicarse con soporte técnico de Internet Claro</t>
-  </si>
-  <si>
-    <t>Todos los canales de atención para clientes Internet Claro</t>
-  </si>
-  <si>
-    <t>Internet Claro soporte: teléfonos, app y atención virtual</t>
-  </si>
-  <si>
-    <t>Atención por WhatsApp</t>
-  </si>
-  <si>
-    <t>Soporte desde Mi Claro</t>
-  </si>
-  <si>
-    <t>Reporte de daños</t>
-  </si>
-  <si>
-    <t>Atención presencial</t>
-  </si>
-  <si>
-    <t>Propuestas con mejor potencial SEO + CTR</t>
-  </si>
-  <si>
-    <t>Estas podrían funcionar especialmente bien para tráfico orgánico:</t>
-  </si>
-  <si>
-    <t>1. Internet Claro: precios, planes y comparación con otros operadores</t>
-  </si>
-  <si>
-    <t>2. ¿Internet Claro está fallando? Soluciones y canales de soporte</t>
-  </si>
-  <si>
-    <t>3. Internet Claro hogar: planes, cobertura y velocidad en Colombia</t>
-  </si>
-  <si>
-    <t>4. Internet Claro vs Movistar y Tigo: cuál conviene más</t>
-  </si>
-  <si>
-    <t>5. Internet Claro lento o sin señal: causas y cómo solucionarlo</t>
-  </si>
-  <si>
-    <t>Recomendación estratégica</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Si quieres posicionar fuerte la keyword </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>“Internet Claro”</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, te conviene hacer un clúster de contenido:</t>
-    </r>
-  </si>
-  <si>
-    <t>Artículo principal:</t>
-  </si>
-  <si>
-    <t>Internet Claro: planes, precios y cobertura</t>
-  </si>
-  <si>
-    <t>Artículos satélite:</t>
-  </si>
-  <si>
-    <t>Internet Claro con fallas</t>
-  </si>
-  <si>
-    <t>Internet Claro vs Movistar</t>
-  </si>
-  <si>
-    <t>Canales de atención Claro</t>
-  </si>
-  <si>
-    <t>Cómo mejorar la velocidad de Internet Claro</t>
-  </si>
-  <si>
-    <t>Eso ayuda muchísimo al enlazado interno y autoridad temática.</t>
   </si>
   <si>
     <t>Comparativa de planes y precios</t>
@@ -1422,58 +1237,68 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF002060"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF333333"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF333333"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF002060"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF002060"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFC0392B"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFE67E22"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF7D6608"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF95A5A6"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1887,7 +1712,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2030,41 +1855,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2080,9 +1874,19 @@
     <xf numFmtId="0" fontId="14" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2095,7 +1899,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2110,8 +1914,17 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2418,7 +2231,7 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:J173"/>
+  <dimension ref="A1:J171"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="92.85546875" bestFit="1" customWidth="1"/>
@@ -2434,90 +2247,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="73" t="s">
         <v>370</v>
       </c>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
+      <c r="B2" s="73"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="71" t="s">
+      <c r="A3" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="72"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="73"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="65"/>
+      <c r="D3" s="66"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="74"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="76"/>
+      <c r="A4" s="67"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="69"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="74"/>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="76"/>
+      <c r="A5" s="67"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="69"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="74"/>
-      <c r="B6" s="75"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="76"/>
+      <c r="A6" s="67"/>
+      <c r="B6" s="68"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="69"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="77"/>
-      <c r="B7" s="78"/>
-      <c r="C7" s="78"/>
-      <c r="D7" s="79"/>
+      <c r="A7" s="70"/>
+      <c r="B7" s="71"/>
+      <c r="C7" s="71"/>
+      <c r="D7" s="72"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="52"/>
-      <c r="D8" s="52"/>
+      <c r="B8" s="73"/>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="70" t="s">
+      <c r="A9" s="76" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="70"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="70"/>
+      <c r="B9" s="76"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="70"/>
-      <c r="B10" s="70"/>
-      <c r="C10" s="70"/>
-      <c r="D10" s="70"/>
+      <c r="A10" s="76"/>
+      <c r="B10" s="76"/>
+      <c r="C10" s="76"/>
+      <c r="D10" s="76"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="33"/>
       <c r="B12" s="33"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="53" t="s">
+      <c r="A13" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="54"/>
+      <c r="B13" s="75"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="80" t="s">
+      <c r="B14" s="59" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2525,7 +2338,7 @@
       <c r="A15" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="80" t="s">
+      <c r="B15" s="59" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2533,7 +2346,7 @@
       <c r="A16" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="80" t="s">
+      <c r="B16" s="59" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2541,7 +2354,7 @@
       <c r="A17" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="80" t="s">
+      <c r="B17" s="59" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2549,7 +2362,7 @@
       <c r="A18" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="80" t="s">
+      <c r="B18" s="59" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2557,7 +2370,7 @@
       <c r="A19" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="80" t="s">
+      <c r="B19" s="59" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2565,7 +2378,7 @@
       <c r="A20" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="80" t="s">
+      <c r="B20" s="59" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2573,7 +2386,7 @@
       <c r="A21" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="80" t="s">
+      <c r="B21" s="59" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2581,7 +2394,7 @@
       <c r="A22" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="80">
+      <c r="B22" s="59">
         <v>151</v>
       </c>
     </row>
@@ -2589,7 +2402,7 @@
       <c r="A23" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="80">
+      <c r="B23" s="59">
         <v>102</v>
       </c>
     </row>
@@ -2597,7 +2410,7 @@
       <c r="A24" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="80">
+      <c r="B24" s="59">
         <v>92</v>
       </c>
     </row>
@@ -2605,7 +2418,7 @@
       <c r="A25" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="80">
+      <c r="B25" s="59">
         <v>85</v>
       </c>
     </row>
@@ -2613,7 +2426,7 @@
       <c r="A26" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="80">
+      <c r="B26" s="59">
         <v>0</v>
       </c>
     </row>
@@ -2621,7 +2434,7 @@
       <c r="A27" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="80">
+      <c r="B27" s="59">
         <v>0</v>
       </c>
     </row>
@@ -2647,7 +2460,7 @@
       <c r="A32" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="59" t="s">
+      <c r="B32" s="53" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2655,7 +2468,7 @@
       <c r="A33" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="58">
+      <c r="B33" s="52">
         <v>42</v>
       </c>
     </row>
@@ -2663,7 +2476,7 @@
       <c r="A34" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B34" s="58">
+      <c r="B34" s="52">
         <v>103</v>
       </c>
     </row>
@@ -2671,7 +2484,7 @@
       <c r="A35" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="B35" s="58">
+      <c r="B35" s="52">
         <v>68</v>
       </c>
     </row>
@@ -2679,7 +2492,7 @@
       <c r="A36" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="58">
+      <c r="B36" s="52">
         <v>66</v>
       </c>
     </row>
@@ -2687,39 +2500,39 @@
       <c r="A37" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B37" s="58">
+      <c r="B37" s="52">
         <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="22" t="s">
-        <v>448</v>
+        <v>394</v>
       </c>
       <c r="B40" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="C40" s="57" t="s">
+      <c r="C40" s="22" t="s">
         <v>372</v>
       </c>
-      <c r="D40" s="40" t="s">
+      <c r="D40" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="E40" s="62" t="s">
+      <c r="E40" s="22" t="s">
         <v>373</v>
       </c>
-      <c r="F40" s="63" t="s">
+      <c r="F40" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="G40" s="57" t="s">
+      <c r="G40" s="22" t="s">
         <v>373</v>
       </c>
-      <c r="H40" s="63" t="s">
+      <c r="H40" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="I40" s="64" t="s">
+      <c r="I40" s="22" t="s">
         <v>374</v>
       </c>
-      <c r="J40" s="63" t="s">
+      <c r="J40" s="22" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2727,31 +2540,31 @@
       <c r="A41" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="65">
+      <c r="B41" s="54">
         <v>100</v>
       </c>
       <c r="C41" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="66">
+      <c r="D41" s="55">
         <v>100</v>
       </c>
-      <c r="E41" s="67" t="s">
+      <c r="E41" s="56" t="s">
         <v>72</v>
       </c>
-      <c r="F41" s="65">
+      <c r="F41" s="54">
         <v>100</v>
       </c>
-      <c r="G41" s="68" t="s">
+      <c r="G41" s="57" t="s">
         <v>72</v>
       </c>
-      <c r="H41" s="65">
+      <c r="H41" s="54">
         <v>100</v>
       </c>
-      <c r="I41" s="68" t="s">
+      <c r="I41" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="J41" s="65">
+      <c r="J41" s="54">
         <v>100</v>
       </c>
     </row>
@@ -2759,31 +2572,31 @@
       <c r="A42" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="B42" s="65">
+      <c r="B42" s="54">
         <v>99.5</v>
       </c>
       <c r="C42" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="D42" s="66">
+      <c r="D42" s="55">
         <v>99.5</v>
       </c>
-      <c r="E42" s="67" t="s">
+      <c r="E42" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="F42" s="65">
+      <c r="F42" s="54">
         <v>99.5</v>
       </c>
-      <c r="G42" s="69" t="s">
+      <c r="G42" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="H42" s="65">
+      <c r="H42" s="54">
         <v>99.5</v>
       </c>
-      <c r="I42" s="69" t="s">
+      <c r="I42" s="58" t="s">
         <v>124</v>
       </c>
-      <c r="J42" s="65">
+      <c r="J42" s="54">
         <v>99.5</v>
       </c>
     </row>
@@ -2791,31 +2604,31 @@
       <c r="A43" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="65">
+      <c r="B43" s="54">
         <v>99.1</v>
       </c>
       <c r="C43" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="D43" s="66">
+      <c r="D43" s="55">
         <v>99.1</v>
       </c>
-      <c r="E43" s="67" t="s">
+      <c r="E43" s="56" t="s">
         <v>74</v>
       </c>
-      <c r="F43" s="65">
+      <c r="F43" s="54">
         <v>99.1</v>
       </c>
-      <c r="G43" s="68" t="s">
+      <c r="G43" s="57" t="s">
         <v>74</v>
       </c>
-      <c r="H43" s="65">
+      <c r="H43" s="54">
         <v>99.1</v>
       </c>
-      <c r="I43" s="68" t="s">
+      <c r="I43" s="57" t="s">
         <v>130</v>
       </c>
-      <c r="J43" s="65">
+      <c r="J43" s="54">
         <v>99.1</v>
       </c>
     </row>
@@ -2823,31 +2636,31 @@
       <c r="A44" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="B44" s="65">
+      <c r="B44" s="54">
         <v>98.6</v>
       </c>
       <c r="C44" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="D44" s="66">
+      <c r="D44" s="55">
         <v>99.1</v>
       </c>
-      <c r="E44" s="67" t="s">
+      <c r="E44" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="F44" s="65">
+      <c r="F44" s="54">
         <v>99.1</v>
       </c>
-      <c r="G44" s="69" t="s">
+      <c r="G44" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="H44" s="65">
+      <c r="H44" s="54">
         <v>99.1</v>
       </c>
-      <c r="I44" s="69" t="s">
+      <c r="I44" s="58" t="s">
         <v>325</v>
       </c>
-      <c r="J44" s="65">
+      <c r="J44" s="54">
         <v>99.1</v>
       </c>
     </row>
@@ -2855,37 +2668,37 @@
       <c r="A45" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="B45" s="65">
+      <c r="B45" s="54">
         <v>98.1</v>
       </c>
       <c r="C45" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="D45" s="66">
+      <c r="D45" s="55">
         <v>98.6</v>
       </c>
-      <c r="E45" s="67" t="s">
+      <c r="E45" s="56" t="s">
         <v>77</v>
       </c>
-      <c r="F45" s="65">
+      <c r="F45" s="54">
         <v>98.6</v>
       </c>
-      <c r="G45" s="68" t="s">
+      <c r="G45" s="57" t="s">
         <v>77</v>
       </c>
-      <c r="H45" s="65">
+      <c r="H45" s="54">
         <v>98.6</v>
       </c>
-      <c r="I45" s="68" t="s">
+      <c r="I45" s="57" t="s">
         <v>326</v>
       </c>
-      <c r="J45" s="65">
+      <c r="J45" s="54">
         <v>98.6</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="22" t="s">
-        <v>449</v>
+        <v>395</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -2920,7 +2733,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="40" t="s">
-        <v>444</v>
+        <v>390</v>
       </c>
       <c r="B55" s="41"/>
       <c r="C55" s="41"/>
@@ -2930,7 +2743,7 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="45" t="s">
-        <v>446</v>
+        <v>392</v>
       </c>
       <c r="B56" s="46"/>
       <c r="C56" s="46"/>
@@ -2938,75 +2751,75 @@
       <c r="E56" s="46"/>
       <c r="F56" s="47"/>
     </row>
-    <row r="57" spans="1:6" ht="54" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="23" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="F57" s="48"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="49" t="s">
-        <v>445</v>
+        <v>391</v>
       </c>
       <c r="F58" s="48"/>
     </row>
-    <row r="59" spans="1:6" ht="27" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="24" t="s">
+        <v>381</v>
+      </c>
+      <c r="F59" s="48"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="23" t="s">
+        <v>382</v>
+      </c>
+      <c r="F60" s="48"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="24" t="s">
         <v>383</v>
       </c>
-      <c r="F59" s="48"/>
-    </row>
-    <row r="60" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A60" s="23" t="s">
+      <c r="F61" s="48"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="23" t="s">
         <v>384</v>
       </c>
-      <c r="F60" s="48"/>
-    </row>
-    <row r="61" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A61" s="24" t="s">
+      <c r="F62" s="48"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="24" t="s">
         <v>385</v>
-      </c>
-      <c r="F61" s="48"/>
-    </row>
-    <row r="62" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A62" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="F62" s="48"/>
-    </row>
-    <row r="63" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A63" s="24" t="s">
-        <v>387</v>
       </c>
       <c r="F63" s="48"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="49" t="s">
-        <v>447</v>
+        <v>393</v>
       </c>
       <c r="F64" s="48"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="F65" s="48"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="23" t="s">
+        <v>387</v>
+      </c>
+      <c r="F66" s="48"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="23" t="s">
+        <v>388</v>
+      </c>
+      <c r="F67" s="48"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="23" t="s">
         <v>389</v>
-      </c>
-      <c r="F65" s="48"/>
-    </row>
-    <row r="66" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A66" s="23" t="s">
-        <v>390</v>
-      </c>
-      <c r="F66" s="48"/>
-    </row>
-    <row r="67" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A67" s="23" t="s">
-        <v>391</v>
-      </c>
-      <c r="F67" s="48"/>
-    </row>
-    <row r="68" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A68" s="23" t="s">
-        <v>392</v>
       </c>
       <c r="B68" s="50"/>
       <c r="C68" s="50"/>
@@ -3015,9 +2828,7 @@
       <c r="F68" s="51"/>
     </row>
     <row r="69" spans="1:6" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A69" s="43" t="s">
-        <v>393</v>
-      </c>
+      <c r="A69" s="43"/>
       <c r="B69" s="44"/>
       <c r="C69" s="44"/>
       <c r="D69" s="44"/>
@@ -3025,326 +2836,190 @@
       <c r="F69" s="44"/>
     </row>
     <row r="70" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A70" s="36" t="s">
-        <v>380</v>
-      </c>
+      <c r="A70" s="36"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="37"/>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>394</v>
-      </c>
-    </row>
     <row r="85" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A85" s="36" t="s">
-        <v>382</v>
-      </c>
+      <c r="A85" s="36"/>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" s="37"/>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" s="37" t="s">
-        <v>395</v>
-      </c>
+      <c r="A87" s="37"/>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" s="37" t="s">
-        <v>396</v>
-      </c>
+      <c r="A88" s="37"/>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" s="37" t="s">
-        <v>397</v>
-      </c>
+      <c r="A89" s="37"/>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" s="37" t="s">
-        <v>398</v>
-      </c>
+      <c r="A90" s="37"/>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" s="37" t="s">
-        <v>399</v>
-      </c>
+      <c r="A91" s="37"/>
     </row>
     <row r="93" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A93" s="36" t="s">
-        <v>388</v>
-      </c>
+      <c r="A93" s="36"/>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" s="37"/>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" s="37" t="s">
-        <v>400</v>
-      </c>
+      <c r="A95" s="37"/>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" s="37" t="s">
-        <v>401</v>
-      </c>
+      <c r="A96" s="37"/>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" s="37" t="s">
-        <v>402</v>
-      </c>
+      <c r="A97" s="37"/>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" s="37" t="s">
-        <v>403</v>
-      </c>
+      <c r="A98" s="37"/>
     </row>
     <row r="102" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A102" s="35" t="s">
-        <v>404</v>
-      </c>
+      <c r="A102" s="35"/>
     </row>
     <row r="104" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A104" s="36" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>405</v>
-      </c>
+      <c r="A104" s="36"/>
     </row>
     <row r="108" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A108" s="36" t="s">
-        <v>382</v>
-      </c>
+      <c r="A108" s="36"/>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" s="37"/>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" s="37" t="s">
-        <v>406</v>
-      </c>
+      <c r="A110" s="37"/>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" s="37" t="s">
-        <v>407</v>
-      </c>
+      <c r="A111" s="37"/>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" s="37" t="s">
-        <v>408</v>
-      </c>
+      <c r="A112" s="37"/>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" s="37" t="s">
-        <v>409</v>
-      </c>
+      <c r="A113" s="37"/>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" s="37" t="s">
-        <v>410</v>
-      </c>
+      <c r="A114" s="37"/>
     </row>
     <row r="116" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A116" s="36" t="s">
-        <v>388</v>
-      </c>
+      <c r="A116" s="36"/>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" s="37"/>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" s="37" t="s">
-        <v>411</v>
-      </c>
+      <c r="A118" s="37"/>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" s="37" t="s">
-        <v>412</v>
-      </c>
+      <c r="A119" s="37"/>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" s="37" t="s">
-        <v>413</v>
-      </c>
+      <c r="A120" s="37"/>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" s="37" t="s">
-        <v>414</v>
-      </c>
+      <c r="A121" s="37"/>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" s="37" t="s">
-        <v>415</v>
-      </c>
+      <c r="A122" s="37"/>
     </row>
     <row r="126" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A126" s="35" t="s">
-        <v>416</v>
-      </c>
+      <c r="A126" s="35"/>
     </row>
     <row r="128" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A128" s="36" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>417</v>
-      </c>
+      <c r="A128" s="36"/>
     </row>
     <row r="132" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A132" s="36" t="s">
-        <v>382</v>
-      </c>
+      <c r="A132" s="36"/>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" s="37"/>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A134" s="37" t="s">
-        <v>418</v>
-      </c>
+      <c r="A134" s="37"/>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A135" s="37" t="s">
-        <v>419</v>
-      </c>
+      <c r="A135" s="37"/>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A136" s="37" t="s">
-        <v>420</v>
-      </c>
+      <c r="A136" s="37"/>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" s="37" t="s">
-        <v>421</v>
-      </c>
+      <c r="A137" s="37"/>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A138" s="37" t="s">
-        <v>422</v>
-      </c>
+      <c r="A138" s="37"/>
     </row>
     <row r="140" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A140" s="36" t="s">
-        <v>388</v>
-      </c>
+      <c r="A140" s="36"/>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" s="37"/>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="37" t="s">
-        <v>423</v>
-      </c>
+      <c r="A142" s="37"/>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" s="37" t="s">
-        <v>424</v>
-      </c>
+      <c r="A143" s="37"/>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A144" s="37" t="s">
-        <v>425</v>
-      </c>
+      <c r="A144" s="37"/>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145" s="37" t="s">
-        <v>426</v>
-      </c>
+      <c r="A145" s="37"/>
     </row>
     <row r="149" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A149" s="34" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>428</v>
-      </c>
+      <c r="A149" s="34"/>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A152" s="37"/>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" s="38" t="s">
-        <v>429</v>
-      </c>
+      <c r="A153" s="38"/>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" s="38" t="s">
-        <v>430</v>
-      </c>
+      <c r="A154" s="38"/>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" s="38" t="s">
-        <v>431</v>
-      </c>
+      <c r="A155" s="38"/>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" s="38" t="s">
-        <v>432</v>
-      </c>
+      <c r="A156" s="38"/>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" s="38" t="s">
-        <v>433</v>
-      </c>
+      <c r="A157" s="38"/>
     </row>
     <row r="161" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A161" s="34" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
-        <v>435</v>
-      </c>
+      <c r="A161" s="34"/>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A164" s="37"/>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A165" s="37" t="s">
-        <v>436</v>
-      </c>
+      <c r="A165" s="37"/>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" s="39" t="s">
-        <v>437</v>
-      </c>
+      <c r="A166" s="39"/>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" s="37" t="s">
-        <v>438</v>
-      </c>
+      <c r="A167" s="37"/>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" s="39" t="s">
-        <v>439</v>
-      </c>
+      <c r="A168" s="39"/>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A169" s="39" t="s">
-        <v>440</v>
-      </c>
+      <c r="A169" s="39"/>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" s="39" t="s">
-        <v>441</v>
-      </c>
+      <c r="A170" s="39"/>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" s="39" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A173" t="s">
-        <v>443</v>
-      </c>
+      <c r="A171" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
chore: actualizar plantilla de excel con nuevos espacios
</commit_message>
<xml_diff>
--- a/PLANTILLA CON INFORME.xlsx
+++ b/PLANTILLA CON INFORME.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="L:\DESCARGAS\PROYECTOS\PROYECTO PREGUNTAS GOOGLE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481FF363-95F8-4CB3-8EC7-EF13300FA1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED280AE-22B3-40D9-9D80-18A01E60ADB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7048" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7067" uniqueCount="400">
   <si>
     <t>Analisis de keyword: Internet claro</t>
   </si>
@@ -1178,30 +1178,9 @@
     <t>Internet Claro: precios y planes para hogar en 2026</t>
   </si>
   <si>
-    <t>¿Cuál es el mejor plan de Internet Claro este año?</t>
-  </si>
-  <si>
-    <t>Internet Claro vs Movistar y Tigo: ¿qué operador conviene más?</t>
-  </si>
-  <si>
-    <t>Planes de Internet Claro: velocidades, precios y beneficios</t>
-  </si>
-  <si>
-    <t>Internet Claro hogar: comparación de planes y cobertura</t>
-  </si>
-  <si>
     <t>Qué incluye cada plan</t>
   </si>
   <si>
-    <t>Diferencias entre fibra óptica y cable</t>
-  </si>
-  <si>
-    <t>Comparativa con Movistar, ETB y Tigo</t>
-  </si>
-  <si>
-    <t>Cómo elegir el mejor plan según tu uso</t>
-  </si>
-  <si>
     <t>Comparativa de planes y precios</t>
   </si>
   <si>
@@ -1218,13 +1197,46 @@
   </si>
   <si>
     <t>EJES ESTRATEGICOS</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2027</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2028</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2029</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2030</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2031</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2032</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2033</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2034</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2035</t>
+  </si>
+  <si>
+    <t>Internet Claro: precios y planes para hogar en 2036</t>
+  </si>
+  <si>
+    <t>Keywords</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1392,8 +1404,14 @@
       <name val="Century Gothic"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1460,8 +1478,14 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="-0.249977111117893"/>
+        <bgColor rgb="FF002060"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -1562,50 +1586,6 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FFD5DDE5"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD5DDE5"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD5DDE5"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFD5DDE5"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD5DDE5"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD5DDE5"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -1628,19 +1608,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD5DDE5"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD5DDE5"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -1708,11 +1675,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD5DDE5"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD5DDE5"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1780,12 +1769,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1829,32 +1812,6 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1864,7 +1821,7 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1887,31 +1844,31 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1926,6 +1883,35 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2247,266 +2233,266 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="73" t="s">
+      <c r="A2" s="59" t="s">
         <v>370</v>
       </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="64" t="s">
+      <c r="A3" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="65"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="66"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="52"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="67"/>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="69"/>
+      <c r="A4" s="53"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="55"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="67"/>
-      <c r="B5" s="68"/>
-      <c r="C5" s="68"/>
-      <c r="D5" s="69"/>
+      <c r="A5" s="53"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="55"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="67"/>
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="69"/>
+      <c r="A6" s="53"/>
+      <c r="B6" s="54"/>
+      <c r="C6" s="54"/>
+      <c r="D6" s="55"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="70"/>
-      <c r="B7" s="71"/>
-      <c r="C7" s="71"/>
-      <c r="D7" s="72"/>
+      <c r="A7" s="56"/>
+      <c r="B7" s="57"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="58"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="73" t="s">
+      <c r="A8" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="73"/>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="59"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="76" t="s">
+      <c r="A9" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="76"/>
-      <c r="D9" s="76"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="76"/>
-      <c r="B10" s="76"/>
-      <c r="C10" s="76"/>
-      <c r="D10" s="76"/>
+      <c r="A10" s="62"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="33"/>
-      <c r="B12" s="33"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="75"/>
+      <c r="B13" s="61"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B14" s="59" t="s">
+      <c r="B14" s="45" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="45" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B16" s="59" t="s">
+      <c r="B16" s="45" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="45" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="59" t="s">
+      <c r="B18" s="45" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="59" t="s">
+      <c r="B19" s="45" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="59" t="s">
+      <c r="B20" s="45" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="59" t="s">
+      <c r="B21" s="45" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="30" t="s">
+      <c r="A22" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="59">
+      <c r="B22" s="45">
         <v>151</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="59">
+      <c r="B23" s="45">
         <v>102</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="30" t="s">
+      <c r="A24" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="59">
+      <c r="B24" s="45">
         <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="59">
+      <c r="B25" s="45">
         <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="59">
+      <c r="B26" s="45">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="59">
+      <c r="B27" s="45">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="30">
         <v>430</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="60" t="s">
+      <c r="A30" s="46" t="s">
         <v>371</v>
       </c>
-      <c r="B30" s="60"/>
+      <c r="B30" s="46"/>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="61"/>
-      <c r="B31" s="61"/>
+      <c r="A31" s="47"/>
+      <c r="B31" s="47"/>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="53" t="s">
+      <c r="B32" s="39" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="26" t="s">
+      <c r="A33" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="52">
+      <c r="B33" s="38">
         <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="27" t="s">
+      <c r="A34" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B34" s="52">
+      <c r="B34" s="38">
         <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B35" s="52">
+      <c r="B35" s="38">
         <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B36" s="52">
+      <c r="B36" s="38">
         <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="B37" s="52">
+      <c r="B37" s="38">
         <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="22" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="B40" s="22" t="s">
         <v>46</v>
@@ -2537,492 +2523,752 @@
       </c>
     </row>
     <row r="41" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="A41" s="25" t="s">
+      <c r="A41" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="B41" s="54">
+      <c r="B41" s="40">
         <v>100</v>
       </c>
-      <c r="C41" s="25" t="s">
+      <c r="C41" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="55">
+      <c r="D41" s="41">
         <v>100</v>
       </c>
-      <c r="E41" s="56" t="s">
+      <c r="E41" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="F41" s="54">
+      <c r="F41" s="40">
         <v>100</v>
       </c>
-      <c r="G41" s="57" t="s">
+      <c r="G41" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="H41" s="54">
+      <c r="H41" s="40">
         <v>100</v>
       </c>
-      <c r="I41" s="57" t="s">
+      <c r="I41" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="J41" s="54">
+      <c r="J41" s="40">
         <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="A42" s="25" t="s">
+      <c r="A42" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B42" s="54">
+      <c r="B42" s="40">
         <v>99.5</v>
       </c>
-      <c r="C42" s="25" t="s">
+      <c r="C42" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="D42" s="55">
+      <c r="D42" s="41">
         <v>99.5</v>
       </c>
-      <c r="E42" s="56" t="s">
+      <c r="E42" s="42" t="s">
         <v>73</v>
       </c>
-      <c r="F42" s="54">
+      <c r="F42" s="40">
         <v>99.5</v>
       </c>
-      <c r="G42" s="58" t="s">
+      <c r="G42" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="H42" s="54">
+      <c r="H42" s="40">
         <v>99.5</v>
       </c>
-      <c r="I42" s="58" t="s">
+      <c r="I42" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="J42" s="54">
+      <c r="J42" s="40">
         <v>99.5</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="A43" s="25" t="s">
+      <c r="A43" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="54">
+      <c r="B43" s="40">
         <v>99.1</v>
       </c>
-      <c r="C43" s="25" t="s">
+      <c r="C43" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="D43" s="55">
+      <c r="D43" s="41">
         <v>99.1</v>
       </c>
-      <c r="E43" s="56" t="s">
+      <c r="E43" s="42" t="s">
         <v>74</v>
       </c>
-      <c r="F43" s="54">
+      <c r="F43" s="40">
         <v>99.1</v>
       </c>
-      <c r="G43" s="57" t="s">
+      <c r="G43" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="H43" s="54">
+      <c r="H43" s="40">
         <v>99.1</v>
       </c>
-      <c r="I43" s="57" t="s">
+      <c r="I43" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="J43" s="54">
+      <c r="J43" s="40">
         <v>99.1</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="A44" s="25" t="s">
+      <c r="A44" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B44" s="54">
+      <c r="B44" s="40">
         <v>98.6</v>
       </c>
-      <c r="C44" s="25" t="s">
+      <c r="C44" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="D44" s="55">
+      <c r="D44" s="41">
         <v>99.1</v>
       </c>
-      <c r="E44" s="56" t="s">
+      <c r="E44" s="42" t="s">
         <v>76</v>
       </c>
-      <c r="F44" s="54">
+      <c r="F44" s="40">
         <v>99.1</v>
       </c>
-      <c r="G44" s="58" t="s">
+      <c r="G44" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="H44" s="54">
+      <c r="H44" s="40">
         <v>99.1</v>
       </c>
-      <c r="I44" s="58" t="s">
+      <c r="I44" s="44" t="s">
         <v>325</v>
       </c>
-      <c r="J44" s="54">
+      <c r="J44" s="40">
         <v>99.1</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="27" x14ac:dyDescent="0.3">
-      <c r="A45" s="25" t="s">
+      <c r="A45" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B45" s="54">
+      <c r="B45" s="40">
         <v>98.1</v>
       </c>
-      <c r="C45" s="25" t="s">
+      <c r="C45" s="23" t="s">
         <v>203</v>
       </c>
-      <c r="D45" s="55">
+      <c r="D45" s="41">
         <v>98.6</v>
       </c>
-      <c r="E45" s="56" t="s">
+      <c r="E45" s="42" t="s">
         <v>77</v>
       </c>
-      <c r="F45" s="54">
+      <c r="F45" s="40">
         <v>98.6</v>
       </c>
-      <c r="G45" s="57" t="s">
+      <c r="G45" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="H45" s="54">
+      <c r="H45" s="40">
         <v>98.6</v>
       </c>
-      <c r="I45" s="57" t="s">
+      <c r="I45" s="43" t="s">
         <v>326</v>
       </c>
-      <c r="J45" s="54">
+      <c r="J45" s="40">
         <v>98.6</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="22" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="23" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" s="23" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="23" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="23" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="63"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="63"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="63"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="63"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="63"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="63"/>
+    </row>
+    <row r="58" spans="1:6" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A58" s="68" t="s">
+        <v>379</v>
+      </c>
+      <c r="B58" s="69"/>
+      <c r="C58" s="69"/>
+      <c r="D58" s="69"/>
+      <c r="E58" s="69"/>
+      <c r="F58" s="69"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="60" t="s">
+        <v>383</v>
+      </c>
+      <c r="B59" s="64"/>
+      <c r="C59" s="64"/>
+      <c r="D59" s="64"/>
+      <c r="E59" s="64"/>
+      <c r="F59" s="61"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="65" t="s">
+        <v>385</v>
+      </c>
+      <c r="B60" s="66"/>
+      <c r="C60" s="66"/>
+      <c r="D60" s="66"/>
+      <c r="E60" s="66"/>
+      <c r="F60" s="67"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="B61" s="70"/>
+      <c r="C61" s="70"/>
+      <c r="D61" s="70"/>
+      <c r="E61" s="70"/>
+      <c r="F61" s="70"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="B62" s="70"/>
+      <c r="C62" s="70"/>
+      <c r="D62" s="70"/>
+      <c r="E62" s="70"/>
+      <c r="F62" s="70"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="B63" s="70"/>
+      <c r="C63" s="70"/>
+      <c r="D63" s="70"/>
+      <c r="E63" s="70"/>
+      <c r="F63" s="70"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="B64" s="70"/>
+      <c r="C64" s="70"/>
+      <c r="D64" s="70"/>
+      <c r="E64" s="70"/>
+      <c r="F64" s="70"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="70" t="s">
+        <v>380</v>
+      </c>
+      <c r="B65" s="70"/>
+      <c r="C65" s="70"/>
+      <c r="D65" s="70"/>
+      <c r="E65" s="70"/>
+      <c r="F65" s="70"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="65" t="s">
+        <v>384</v>
+      </c>
+      <c r="B66" s="66"/>
+      <c r="C66" s="66"/>
+      <c r="D66" s="66"/>
+      <c r="E66" s="66"/>
+      <c r="F66" s="67"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="71" t="s">
+        <v>381</v>
+      </c>
+      <c r="B67" s="71"/>
+      <c r="C67" s="71"/>
+      <c r="D67" s="71"/>
+      <c r="E67" s="71"/>
+      <c r="F67" s="71"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="71" t="s">
+        <v>389</v>
+      </c>
+      <c r="B68" s="71"/>
+      <c r="C68" s="71"/>
+      <c r="D68" s="71"/>
+      <c r="E68" s="71"/>
+      <c r="F68" s="71"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="71" t="s">
+        <v>390</v>
+      </c>
+      <c r="B69" s="71"/>
+      <c r="C69" s="71"/>
+      <c r="D69" s="71"/>
+      <c r="E69" s="71"/>
+      <c r="F69" s="71"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="71" t="s">
+        <v>391</v>
+      </c>
+      <c r="B70" s="71"/>
+      <c r="C70" s="71"/>
+      <c r="D70" s="71"/>
+      <c r="E70" s="71"/>
+      <c r="F70" s="71"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="71" t="s">
+        <v>392</v>
+      </c>
+      <c r="B71" s="71"/>
+      <c r="C71" s="71"/>
+      <c r="D71" s="71"/>
+      <c r="E71" s="71"/>
+      <c r="F71" s="71"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="71" t="s">
+        <v>393</v>
+      </c>
+      <c r="B72" s="71"/>
+      <c r="C72" s="71"/>
+      <c r="D72" s="71"/>
+      <c r="E72" s="71"/>
+      <c r="F72" s="71"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="71" t="s">
+        <v>394</v>
+      </c>
+      <c r="B73" s="71"/>
+      <c r="C73" s="71"/>
+      <c r="D73" s="71"/>
+      <c r="E73" s="71"/>
+      <c r="F73" s="71"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="71" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="25" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="25" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="25" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="25" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A54" s="43" t="s">
-        <v>379</v>
-      </c>
-      <c r="B54" s="44"/>
-      <c r="C54" s="44"/>
-      <c r="D54" s="44"/>
-      <c r="E54" s="44"/>
-      <c r="F54" s="44"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="40" t="s">
-        <v>390</v>
-      </c>
-      <c r="B55" s="41"/>
-      <c r="C55" s="41"/>
-      <c r="D55" s="41"/>
-      <c r="E55" s="41"/>
-      <c r="F55" s="42"/>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="45" t="s">
-        <v>392</v>
-      </c>
-      <c r="B56" s="46"/>
-      <c r="C56" s="46"/>
-      <c r="D56" s="46"/>
-      <c r="E56" s="46"/>
-      <c r="F56" s="47"/>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="23" t="s">
-        <v>380</v>
-      </c>
-      <c r="F57" s="48"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="49" t="s">
-        <v>391</v>
-      </c>
-      <c r="F58" s="48"/>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="24" t="s">
-        <v>381</v>
-      </c>
-      <c r="F59" s="48"/>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="23" t="s">
+      <c r="B74" s="71"/>
+      <c r="C74" s="71"/>
+      <c r="D74" s="71"/>
+      <c r="E74" s="71"/>
+      <c r="F74" s="71"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="71" t="s">
+        <v>396</v>
+      </c>
+      <c r="B75" s="71"/>
+      <c r="C75" s="71"/>
+      <c r="D75" s="71"/>
+      <c r="E75" s="71"/>
+      <c r="F75" s="71"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="71" t="s">
+        <v>397</v>
+      </c>
+      <c r="B76" s="71"/>
+      <c r="C76" s="71"/>
+      <c r="D76" s="71"/>
+      <c r="E76" s="71"/>
+      <c r="F76" s="71"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="71" t="s">
+        <v>398</v>
+      </c>
+      <c r="B77" s="71"/>
+      <c r="C77" s="71"/>
+      <c r="D77" s="71"/>
+      <c r="E77" s="71"/>
+      <c r="F77" s="71"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="65" t="s">
+        <v>386</v>
+      </c>
+      <c r="B78" s="66"/>
+      <c r="C78" s="66"/>
+      <c r="D78" s="66"/>
+      <c r="E78" s="66"/>
+      <c r="F78" s="66"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="70" t="s">
         <v>382</v>
       </c>
-      <c r="F60" s="48"/>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="24" t="s">
-        <v>383</v>
-      </c>
-      <c r="F61" s="48"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="23" t="s">
-        <v>384</v>
-      </c>
-      <c r="F62" s="48"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="24" t="s">
-        <v>385</v>
-      </c>
-      <c r="F63" s="48"/>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="49" t="s">
-        <v>393</v>
-      </c>
-      <c r="F64" s="48"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="F65" s="48"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="23" t="s">
-        <v>387</v>
-      </c>
-      <c r="F66" s="48"/>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="23" t="s">
-        <v>388</v>
-      </c>
-      <c r="F67" s="48"/>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="23" t="s">
-        <v>389</v>
-      </c>
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-      <c r="D68" s="50"/>
-      <c r="E68" s="50"/>
-      <c r="F68" s="51"/>
-    </row>
-    <row r="69" spans="1:6" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A69" s="43"/>
-      <c r="B69" s="44"/>
-      <c r="C69" s="44"/>
-      <c r="D69" s="44"/>
-      <c r="E69" s="44"/>
-      <c r="F69" s="44"/>
-    </row>
-    <row r="70" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A70" s="36"/>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="37"/>
-    </row>
-    <row r="85" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A85" s="36"/>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" s="37"/>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" s="37"/>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" s="37"/>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" s="37"/>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" s="37"/>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" s="37"/>
-    </row>
-    <row r="93" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A93" s="36"/>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" s="37"/>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" s="37"/>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" s="37"/>
+      <c r="B79" s="70"/>
+      <c r="C79" s="70"/>
+      <c r="D79" s="70"/>
+      <c r="E79" s="70"/>
+      <c r="F79" s="70"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B80" s="70"/>
+      <c r="C80" s="70"/>
+      <c r="D80" s="70"/>
+      <c r="E80" s="70"/>
+      <c r="F80" s="70"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B81" s="70"/>
+      <c r="C81" s="70"/>
+      <c r="D81" s="70"/>
+      <c r="E81" s="70"/>
+      <c r="F81" s="70"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B82" s="70"/>
+      <c r="C82" s="70"/>
+      <c r="D82" s="70"/>
+      <c r="E82" s="70"/>
+      <c r="F82" s="70"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B83" s="70"/>
+      <c r="C83" s="70"/>
+      <c r="D83" s="70"/>
+      <c r="E83" s="70"/>
+      <c r="F83" s="70"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B84" s="70"/>
+      <c r="C84" s="70"/>
+      <c r="D84" s="70"/>
+      <c r="E84" s="70"/>
+      <c r="F84" s="70"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B85" s="70"/>
+      <c r="C85" s="70"/>
+      <c r="D85" s="70"/>
+      <c r="E85" s="70"/>
+      <c r="F85" s="70"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B86" s="70"/>
+      <c r="C86" s="70"/>
+      <c r="D86" s="70"/>
+      <c r="E86" s="70"/>
+      <c r="F86" s="70"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B87" s="70"/>
+      <c r="C87" s="70"/>
+      <c r="D87" s="70"/>
+      <c r="E87" s="70"/>
+      <c r="F87" s="70"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B88" s="70"/>
+      <c r="C88" s="70"/>
+      <c r="D88" s="70"/>
+      <c r="E88" s="70"/>
+      <c r="F88" s="70"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B89" s="70"/>
+      <c r="C89" s="70"/>
+      <c r="D89" s="70"/>
+      <c r="E89" s="70"/>
+      <c r="F89" s="70"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="70" t="s">
+        <v>382</v>
+      </c>
+      <c r="B90" s="70"/>
+      <c r="C90" s="70"/>
+      <c r="D90" s="70"/>
+      <c r="E90" s="70"/>
+      <c r="F90" s="70"/>
+    </row>
+    <row r="91" spans="1:6" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A91" s="72" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" s="73"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="73"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="73"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" s="73"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" s="73"/>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" s="37"/>
+      <c r="A97" s="73"/>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" s="37"/>
-    </row>
-    <row r="102" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A102" s="35"/>
+      <c r="A98" s="73"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="73"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="73"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="73"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="73"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="73"/>
     </row>
     <row r="104" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A104" s="36"/>
+      <c r="A104" s="34"/>
     </row>
     <row r="108" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A108" s="36"/>
+      <c r="A108" s="34"/>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A109" s="37"/>
+      <c r="A109" s="35"/>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" s="37"/>
+      <c r="A110" s="35"/>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" s="37"/>
+      <c r="A111" s="35"/>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" s="37"/>
+      <c r="A112" s="35"/>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" s="37"/>
+      <c r="A113" s="35"/>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" s="37"/>
+      <c r="A114" s="35"/>
     </row>
     <row r="116" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A116" s="36"/>
+      <c r="A116" s="34"/>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A117" s="37"/>
+      <c r="A117" s="35"/>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" s="37"/>
+      <c r="A118" s="35"/>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" s="37"/>
+      <c r="A119" s="35"/>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" s="37"/>
+      <c r="A120" s="35"/>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" s="37"/>
+      <c r="A121" s="35"/>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" s="37"/>
+      <c r="A122" s="35"/>
     </row>
     <row r="126" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A126" s="35"/>
+      <c r="A126" s="33"/>
     </row>
     <row r="128" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A128" s="36"/>
+      <c r="A128" s="34"/>
     </row>
     <row r="132" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A132" s="36"/>
+      <c r="A132" s="34"/>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A133" s="37"/>
+      <c r="A133" s="35"/>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A134" s="37"/>
+      <c r="A134" s="35"/>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A135" s="37"/>
+      <c r="A135" s="35"/>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A136" s="37"/>
+      <c r="A136" s="35"/>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A137" s="37"/>
+      <c r="A137" s="35"/>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A138" s="37"/>
+      <c r="A138" s="35"/>
     </row>
     <row r="140" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A140" s="36"/>
+      <c r="A140" s="34"/>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A141" s="37"/>
+      <c r="A141" s="35"/>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A142" s="37"/>
+      <c r="A142" s="35"/>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A143" s="37"/>
+      <c r="A143" s="35"/>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A144" s="37"/>
+      <c r="A144" s="35"/>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A145" s="37"/>
+      <c r="A145" s="35"/>
     </row>
     <row r="149" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A149" s="34"/>
+      <c r="A149" s="32"/>
     </row>
     <row r="152" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A152" s="37"/>
+      <c r="A152" s="35"/>
     </row>
     <row r="153" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A153" s="38"/>
+      <c r="A153" s="36"/>
     </row>
     <row r="154" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A154" s="38"/>
+      <c r="A154" s="36"/>
     </row>
     <row r="155" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A155" s="38"/>
+      <c r="A155" s="36"/>
     </row>
     <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" s="38"/>
+      <c r="A156" s="36"/>
     </row>
     <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" s="38"/>
+      <c r="A157" s="36"/>
     </row>
     <row r="161" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A161" s="34"/>
+      <c r="A161" s="32"/>
     </row>
     <row r="164" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A164" s="37"/>
+      <c r="A164" s="35"/>
     </row>
     <row r="165" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A165" s="37"/>
+      <c r="A165" s="35"/>
     </row>
     <row r="166" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A166" s="39"/>
+      <c r="A166" s="37"/>
     </row>
     <row r="167" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A167" s="37"/>
+      <c r="A167" s="35"/>
     </row>
     <row r="168" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A168" s="39"/>
+      <c r="A168" s="37"/>
     </row>
     <row r="169" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A169" s="39"/>
+      <c r="A169" s="37"/>
     </row>
     <row r="170" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A170" s="39"/>
+      <c r="A170" s="37"/>
     </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A171" s="39"/>
+      <c r="A171" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="40">
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="A89:F89"/>
+    <mergeCell ref="A90:F90"/>
+    <mergeCell ref="A83:F83"/>
+    <mergeCell ref="A84:F84"/>
+    <mergeCell ref="A85:F85"/>
+    <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="A78:F78"/>
+    <mergeCell ref="A79:F79"/>
+    <mergeCell ref="A80:F80"/>
+    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A69:F69"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A61:F61"/>
+    <mergeCell ref="A62:F62"/>
     <mergeCell ref="A30:B31"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A3:D7"/>
@@ -3031,6 +3277,7 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A9:D10"/>
   </mergeCells>
+  <phoneticPr fontId="24" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>